<commit_message>
feat: manage extraction filters in Excel
</commit_message>
<xml_diff>
--- a/extraction_plan.xlsx
+++ b/extraction_plan.xlsx
@@ -8,15 +8,15 @@
   </bookViews>
   <sheets>
     <sheet name="抽取计划" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="数据源" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="字段映射" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="字段映射" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="过滤条件" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="填写说明" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'抽取计划'!$A$1:$N$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'数据源'!$A$1:$I$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'字段映射'!$A$1:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'填写说明'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'抽取计划'!$A$1:$M$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'字段映射'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'过滤条件'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'填写说明'!$A$1:$B$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,23 +433,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,12 +464,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>数据源ID</t>
+          <t>源对象</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>源对象</t>
+          <t>表头行</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -495,30 +494,25 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>过滤条件</t>
+          <t>输出格式</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>输出格式</t>
+          <t>输出路径</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>输出路径</t>
+          <t>批次大小</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>批次大小</t>
+          <t>负责人</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>负责人</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -537,14 +531,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>local_demo</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
           <t>orders</t>
         </is>
       </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>增量</t>
@@ -567,35 +559,30 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>status = 'paid'</t>
+          <t>csv</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>csv</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
           <t>./output/orders.csv</t>
         </is>
       </c>
-      <c r="L2" t="n">
+      <c r="K2" t="n">
         <v>10000</v>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>数据组</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>数据组</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
           <t>示例任务，启用前请修改</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N2"/>
+  <autoFilter ref="A1:M2"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"是,否"</formula1>
@@ -603,7 +590,7 @@
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"全量,增量"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"csv,jsonl,xlsx"</formula1>
     </dataValidation>
   </dataValidations>
@@ -612,165 +599,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>数据源ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>类型</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>连接地址</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>端口</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>数据库</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Schema</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>用户名</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>密码环境变量</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>扩展参数</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>local_demo</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>sqlite</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>./data/demo.db</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>excel_demo</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>excel</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>./data/source.xlsx</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>{"header_row": 1}</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>json_demo</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>./data/source.json</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>{"encoding": "utf-8"}</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:I4"/>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"sqlite,excel,json"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -912,13 +740,181 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>任务ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>条件组</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>条件序号</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>运算符</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>值1</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>值2</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>demo_orders</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>同组内为 AND</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>demo_orders</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>&gt;=</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>100</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>demo_orders</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>华东,华南</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>不同组之间为 OR</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H4"/>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"=,!=,&gt;,&gt;=,&lt;,&lt;=,IN,NOT IN,BETWEEN,LIKE,NOT LIKE,IS NULL,IS NOT NULL"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -945,7 +941,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>填写数据源和任务 → validate 校验 → preview 预览 SQL → run 执行抽取</t>
+          <t>填写任务 → validate 校验 → preview 预览 SQL → run 时指定源 Excel 执行抽取</t>
         </is>
       </c>
     </row>
@@ -969,7 +965,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SQLite: 表/视图名；Excel: 工作表名；JSON: 根对象中的数组键，根为数组时可填 data</t>
+          <t>Excel 工作表名称，支持中文</t>
         </is>
       </c>
     </row>
@@ -1024,41 +1020,53 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>密码</t>
+          <t>过滤条件</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>只填写环境变量名，例如 PD_PROD_PASSWORD，禁止把密码明文放进 Excel</t>
+          <t>一行一个条件；同一条件组内使用 AND，不同条件组之间使用 OR；没有记录表示不过滤</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>当前连接器</t>
+          <t>条件值</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>sqlite、excel、json</t>
+          <t>IN/NOT IN 的值1使用英文逗号分隔；BETWEEN 同时填写值1和值2；IS NULL 类无需填写值</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Excel数据源</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>执行 run 命令时传入；表头行从 1 开始计数</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>输出格式</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>csv、jsonl 或 xlsx；相对路径以当前工作目录为基准</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
+  <autoFilter ref="A1:B12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: support joins across Excel sheets
</commit_message>
<xml_diff>
--- a/extraction_plan.xlsx
+++ b/extraction_plan.xlsx
@@ -8,15 +8,19 @@
   </bookViews>
   <sheets>
     <sheet name="抽取计划" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="字段映射" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="过滤条件" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="填写说明" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="数据对象" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="关联关系" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="字段映射" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="过滤条件" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="填写说明" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'抽取计划'!$A$1:$M$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'字段映射'!$A$1:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'过滤条件'!$A$1:$H$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'填写说明'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'抽取计划'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'数据对象'!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'关联关系'!$A$1:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'字段映射'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'过滤条件'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'填写说明'!$A$1:$B$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,22 +437,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -464,55 +466,45 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>源对象</t>
+          <t>抽取模式</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>表头行</t>
+          <t>增量字段</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>抽取模式</t>
+          <t>开始值</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>增量字段</t>
+          <t>结束值</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>开始值</t>
+          <t>输出格式</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>结束值</t>
+          <t>输出路径</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>输出格式</t>
+          <t>批次大小</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>输出路径</t>
+          <t>负责人</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>批次大小</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>负责人</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -531,66 +523,58 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>orders</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1</v>
+          <t>增量</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>o.updated_at</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>增量</t>
+          <t>${START_TIME}</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>${END_TIME}</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>${START_TIME}</t>
+          <t>csv</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>${END_TIME}</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>csv</t>
-        </is>
+          <t>./output/orders.csv</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>10000</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>./output/orders.csv</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>10000</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
           <t>数据组</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>示例任务，启用前请修改</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M2"/>
+  <autoFilter ref="A1:K2"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"是,否"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"全量,增量"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"csv,jsonl,xlsx"</formula1>
     </dataValidation>
   </dataValidations>
@@ -599,6 +583,227 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>任务ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sheet名称</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>对象别名</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>表头行</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>是否主表</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>demo_orders</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>订单</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>主表</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>demo_orders</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>订单明细</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>关联表示例</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F3"/>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"是,否"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>任务ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>关联顺序</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>关联类型</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>左侧字段</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>右侧对象</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>右侧字段</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>demo_orders</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>LEFT JOIN</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>o.order_id</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>i.order_id</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>同一关联顺序可配置多个 ON 条件</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G2"/>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"INNER JOIN,LEFT JOIN"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -661,7 +866,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>o.order_id</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -688,7 +893,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>i.amount</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -715,7 +920,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>o.updated_at</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -740,7 +945,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -815,7 +1020,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>o.status</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -849,7 +1054,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>i.amount</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -877,7 +1082,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>o.region</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -908,13 +1113,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -960,113 +1165,125 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>源对象</t>
+          <t>数据对象</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Excel 工作表名称，支持中文</t>
+          <t>每个任务配置一个或多个 Sheet 和对象别名，并且必须且只能有一个主表</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>抽取模式</t>
+          <t>关联关系</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>全量或增量；增量任务必须填写增量字段</t>
+          <t>支持 INNER JOIN 和 LEFT JOIN；相同关联顺序的多行表示多个 AND 连接条件</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>开始值/结束值</t>
+          <t>抽取模式</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>增量区间为 [开始值, 结束值)；支持 ${ENV_NAME} 环境变量占位符</t>
+          <t>全量或增量；增量任务必须填写增量字段</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>过滤条件</t>
+          <t>开始值/结束值</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>可选的 SQL 条件，不要填写 WHERE；内容会原样拼接，执行前务必 preview</t>
+          <t>增量区间为 [开始值, 结束值)；支持 ${ENV_NAME} 环境变量占位符</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>字段映射</t>
+          <t>过滤条件</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>不配置时抽取 *；转换表达式是源端 SQL 表达式，目标字段是输出列名</t>
+          <t>可选的 SQL 条件，不要填写 WHERE；内容会原样拼接，执行前务必 preview</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>过滤条件</t>
+          <t>字段映射</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>一行一个条件；同一条件组内使用 AND，不同条件组之间使用 OR；没有记录表示不过滤</t>
+          <t>源字段使用 别名.字段；不配置时抽取 *；转换表达式是内部 SQL 表达式</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>条件值</t>
+          <t>过滤条件</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IN/NOT IN 的值1使用英文逗号分隔；BETWEEN 同时填写值1和值2；IS NULL 类无需填写值</t>
+          <t>一行一个条件；同一条件组内使用 AND，不同条件组之间使用 OR；没有记录表示不过滤</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Excel数据源</t>
+          <t>条件值</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>执行 run 命令时传入；表头行从 1 开始计数</t>
+          <t>IN/NOT IN 的值1使用英文逗号分隔；BETWEEN 同时填写值1和值2；IS NULL 类无需填写值</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Excel数据源</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>执行 run 命令时传入同一个工作簿；每个数据对象的表头行从 1 开始计数</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>输出格式</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>csv、jsonl 或 xlsx；相对路径以当前工作目录为基准</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B12"/>
+  <autoFilter ref="A1:B13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: migrate to ExcelFlow pandas package
</commit_message>
<xml_diff>
--- a/extraction_plan.xlsx
+++ b/extraction_plan.xlsx
@@ -15,12 +15,12 @@
     <sheet name="填写说明" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'抽取计划'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'抽取计划'!$A$1:$J$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'数据对象'!$A$1:$F$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'关联关系'!$A$1:$G$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'字段映射'!$A$1:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'过滤条件'!$A$1:$H$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'填写说明'!$A$1:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'字段映射'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'过滤条件'!$A$1:$H$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'填写说明'!$A$1:$B$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -448,9 +448,8 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,15 +495,10 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>批次大小</t>
+          <t>负责人</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>负责人</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -551,22 +545,19 @@
           <t>./output/orders.csv</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>10000</v>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>数据组</t>
+        </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>数据组</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>示例任务，启用前请修改</t>
+          <t>示例任务</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:J2"/>
   <dataValidations count="3">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"是,否"</formula1>
@@ -687,7 +678,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>关联表示例</t>
+          <t>关联表</t>
         </is>
       </c>
     </row>
@@ -788,7 +779,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>同一关联顺序可配置多个 ON 条件</t>
+          <t>相同顺序可配置多个关联字段</t>
         </is>
       </c>
     </row>
@@ -809,14 +800,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
@@ -891,14 +882,10 @@
           <t>demo_orders</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>i.amount</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>total_amount</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -906,41 +893,22 @@
           <t>decimal</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>coalesce(i.quantity, 0) * coalesce(i.unit_price, 0)</t>
+        </is>
+      </c>
       <c r="F3" t="n">
         <v>2</v>
       </c>
-      <c r="G3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>demo_orders</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>o.updated_at</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>updated_at</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>datetime</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Pandas安全表达式</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:G3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -951,7 +919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1036,74 +1004,12 @@
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>同组内为 AND</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>demo_orders</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>i.amount</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>&gt;=</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>100</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>demo_orders</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>o.region</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>华东,华南</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>不同组之间为 OR</t>
+          <t>组内AND，组间OR</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H4"/>
+  <autoFilter ref="A1:H2"/>
   <dataValidations count="1">
     <dataValidation sqref="E2:E5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"=,!=,&gt;,&gt;=,&lt;,&lt;=,IN,NOT IN,BETWEEN,LIKE,NOT LIKE,IS NULL,IS NOT NULL"</formula1>
@@ -1119,7 +1025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1141,149 +1047,89 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>使用流程</t>
+          <t>执行引擎</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>填写任务 → validate 校验 → preview 预览 SQL → run 时指定源 Excel 执行抽取</t>
+          <t>Pandas；计划会被解释为 read_excel、merge、布尔过滤和 Series 运算，不执行 SQL 或 eval</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>启用</t>
+          <t>数据对象</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>是/否；只有“是”的任务允许执行</t>
+          <t>每个任务必须且只能有一个主表；同一源 Excel 可配置多个 Sheet</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>数据对象</t>
+          <t>关联关系</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>每个任务配置一个或多个 Sheet 和对象别名，并且必须且只能有一个主表</t>
+          <t>支持 INNER JOIN 和 LEFT JOIN；相同关联顺序的多行组成复合关联键</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>关联关系</t>
+          <t>字段</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>支持 INNER JOIN 和 LEFT JOIN；相同关联顺序的多行表示多个 AND 连接条件</t>
+          <t>增量、映射、过滤和表达式字段使用 别名.字段</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>抽取模式</t>
+          <t>转换表达式</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>全量或增量；增量任务必须填写增量字段</t>
+          <t>支持 + - * / %、coalesce、abs、round，例如 coalesce(i.quantity, 0) * i.price</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>开始值/结束值</t>
+          <t>过滤条件</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>增量区间为 [开始值, 结束值)；支持 ${ENV_NAME} 环境变量占位符</t>
+          <t>同组内 AND，不同组之间 OR；IN 值用英文逗号分隔</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>过滤条件</t>
+          <t>增量范围</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>可选的 SQL 条件，不要填写 WHERE；内容会原样拼接，执行前务必 preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>字段映射</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>源字段使用 别名.字段；不配置时抽取 *；转换表达式是内部 SQL 表达式</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>过滤条件</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>一行一个条件；同一条件组内使用 AND，不同条件组之间使用 OR；没有记录表示不过滤</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>条件值</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>IN/NOT IN 的值1使用英文逗号分隔；BETWEEN 同时填写值1和值2；IS NULL 类无需填写值</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Excel数据源</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>执行 run 命令时传入同一个工作簿；每个数据对象的表头行从 1 开始计数</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>输出格式</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>csv、jsonl 或 xlsx；相对路径以当前工作目录为基准</t>
+          <t>左闭右开 [开始值, 结束值)，支持 ${ENV_NAME}</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B13"/>
+  <autoFilter ref="A1:B8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: simplify extraction task configuration
</commit_message>
<xml_diff>
--- a/extraction_plan.xlsx
+++ b/extraction_plan.xlsx
@@ -15,7 +15,7 @@
     <sheet name="填写说明" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'抽取计划'!$A$1:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'抽取计划'!$A$1:$C$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'数据对象'!$A$1:$F$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'关联关系'!$A$1:$G$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'字段映射'!$A$1:$G$3</definedName>
@@ -437,19 +437,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,41 +458,6 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>抽取模式</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>增量字段</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>开始值</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>结束值</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>输出格式</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>输出路径</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>负责人</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
           <t>备注</t>
         </is>
       </c>
@@ -517,56 +475,15 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>增量</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>o.updated_at</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>${START_TIME}</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>${END_TIME}</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>csv</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>./output/orders.csv</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>数据组</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
           <t>示例任务</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J2"/>
-  <dataValidations count="3">
+  <autoFilter ref="A1:C2"/>
+  <dataValidations count="1">
     <dataValidation sqref="B2:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"是,否"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"全量,增量"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"csv,jsonl,xlsx"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1088,7 +1005,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>增量、映射、过滤和表达式字段使用 别名.字段</t>
+          <t>映射、过滤和表达式字段使用 别名.字段</t>
         </is>
       </c>
     </row>
@@ -1119,12 +1036,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>增量范围</t>
+          <t>输出</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>左闭右开 [开始值, 结束值)，支持 ${ENV_NAME}</t>
+          <t>执行 run 时分别指定输出格式（csv/jsonl/xlsx）和输出路径</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add guided examples and type selection
</commit_message>
<xml_diff>
--- a/extraction_plan.xlsx
+++ b/extraction_plan.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'关联关系'!$A$1:$G$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'字段映射'!$A$1:$G$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'过滤条件'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'填写说明'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'填写说明'!$A$1:$B$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -826,6 +826,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G3"/>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"integer,decimal,string,datetime"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -942,7 +947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1024,29 +1029,41 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>过滤条件</t>
+          <t>目标类型</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>同组内 AND，不同组之间 OR；IN 值用英文逗号分隔</t>
+          <t>从下拉框选择 integer、decimal、string 或 datetime，执行时会转换输出列类型</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>过滤条件</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>同组内 AND，不同组之间 OR；IN 值用英文逗号分隔</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>输出</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>执行 run 时分别指定输出格式（csv/jsonl/xlsx）和输出路径</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>